<commit_message>
ADD: generated invoice files
</commit_message>
<xml_diff>
--- a/SPLIT_COMPANY_DATA/RESULT/companies_result/ОБЩИНА АКСАКОВО % 1/ОБЩИНА АКСАКОВО % 1.xlsx
+++ b/SPLIT_COMPANY_DATA/RESULT/companies_result/ОБЩИНА АКСАКОВО % 1/ОБЩИНА АКСАКОВО % 1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="104">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="97">
   <si>
     <t>Дата</t>
   </si>
@@ -55,259 +55,238 @@
     <t>Billing_Document</t>
   </si>
   <si>
-    <t>2026-06-16</t>
-  </si>
-  <si>
-    <t>2026-06-17</t>
-  </si>
-  <si>
-    <t>2026-06-18</t>
-  </si>
-  <si>
-    <t>2026-06-19</t>
-  </si>
-  <si>
-    <t>2026-06-20</t>
-  </si>
-  <si>
-    <t>2026-06-22</t>
-  </si>
-  <si>
-    <t>2026-06-23</t>
-  </si>
-  <si>
-    <t>2026-06-24</t>
-  </si>
-  <si>
-    <t>2026-06-25</t>
-  </si>
-  <si>
-    <t>2026-06-26</t>
-  </si>
-  <si>
-    <t>2026-06-29</t>
-  </si>
-  <si>
-    <t>2026-06-30</t>
-  </si>
-  <si>
-    <t>Варна Порт</t>
-  </si>
-  <si>
-    <t>Варна Варненчик</t>
-  </si>
-  <si>
-    <t>София България</t>
-  </si>
-  <si>
-    <t>Търговище</t>
-  </si>
-  <si>
-    <t>В9933СМ</t>
+    <t>2026-07-01</t>
+  </si>
+  <si>
+    <t>2026-07-02</t>
+  </si>
+  <si>
+    <t>2026-07-03</t>
+  </si>
+  <si>
+    <t>2026-07-06</t>
+  </si>
+  <si>
+    <t>2026-07-07</t>
+  </si>
+  <si>
+    <t>2026-07-08</t>
+  </si>
+  <si>
+    <t>2026-07-09</t>
+  </si>
+  <si>
+    <t>2026-07-10</t>
+  </si>
+  <si>
+    <t>2026-07-13</t>
+  </si>
+  <si>
+    <t>2026-07-14</t>
+  </si>
+  <si>
+    <t>2026-07-15</t>
+  </si>
+  <si>
+    <t>1147 Варна Ситроен</t>
+  </si>
+  <si>
+    <t>1158 Варна Чайка</t>
+  </si>
+  <si>
+    <t>1146 Варна Сливница</t>
+  </si>
+  <si>
+    <t>В2278РВ</t>
   </si>
   <si>
     <t>В6431НР</t>
   </si>
   <si>
+    <t>В6613КС</t>
+  </si>
+  <si>
+    <t>В4239ВТ</t>
+  </si>
+  <si>
+    <t>В8636СТ</t>
+  </si>
+  <si>
+    <t>В5089РВ</t>
+  </si>
+  <si>
+    <t>В7341ВС</t>
+  </si>
+  <si>
+    <t>В1283НТ</t>
+  </si>
+  <si>
+    <t>В2429ТТ</t>
+  </si>
+  <si>
+    <t>B6947НТ</t>
+  </si>
+  <si>
+    <t>В5116РС</t>
+  </si>
+  <si>
+    <t>В5163ХВ</t>
+  </si>
+  <si>
     <t>В6476ВС</t>
   </si>
   <si>
-    <t>B6947НТ</t>
-  </si>
-  <si>
-    <t>В5089РВ</t>
-  </si>
-  <si>
-    <t>В6613КС</t>
-  </si>
-  <si>
-    <t>В2429ТТ</t>
+    <t>В5654ВН</t>
+  </si>
+  <si>
+    <t>В6915ВХ</t>
+  </si>
+  <si>
+    <t>В5328РМ</t>
   </si>
   <si>
     <t>В4692РС</t>
   </si>
   <si>
-    <t>В6196РС</t>
-  </si>
-  <si>
-    <t>В7341ВС</t>
-  </si>
-  <si>
-    <t>В5654ВН</t>
-  </si>
-  <si>
-    <t>В1293НН</t>
-  </si>
-  <si>
-    <t>В5328РМ</t>
-  </si>
-  <si>
-    <t>В5163ХВ</t>
-  </si>
-  <si>
-    <t>В4239ВТ</t>
-  </si>
-  <si>
-    <t>В1283НТ</t>
-  </si>
-  <si>
-    <t>В8636СТ</t>
-  </si>
-  <si>
-    <t>78970155027722176</t>
+    <t>78970155027722226</t>
   </si>
   <si>
     <t>78970155027722358</t>
   </si>
   <si>
+    <t>78970155027722168</t>
+  </si>
+  <si>
+    <t>78970155027722325</t>
+  </si>
+  <si>
+    <t>78970155027722184</t>
+  </si>
+  <si>
+    <t>78970155027722382</t>
+  </si>
+  <si>
+    <t>78970155027722390</t>
+  </si>
+  <si>
+    <t>78970155027722333</t>
+  </si>
+  <si>
+    <t>78970155027722408</t>
+  </si>
+  <si>
+    <t>78970155027722416</t>
+  </si>
+  <si>
+    <t>78970155027722267</t>
+  </si>
+  <si>
+    <t>78970155027722374</t>
+  </si>
+  <si>
     <t>78970155027722283</t>
   </si>
   <si>
-    <t>78970155027722416</t>
-  </si>
-  <si>
-    <t>78970155027722382</t>
-  </si>
-  <si>
-    <t>78970155027722168</t>
-  </si>
-  <si>
-    <t>78970155027722408</t>
+    <t>78970155027722309</t>
+  </si>
+  <si>
+    <t>78970155027722291</t>
+  </si>
+  <si>
+    <t>78970155027722259</t>
   </si>
   <si>
     <t>78970155027722234</t>
   </si>
   <si>
-    <t>78970155027722424</t>
-  </si>
-  <si>
-    <t>78970155027722390</t>
-  </si>
-  <si>
-    <t>78970155027722309</t>
-  </si>
-  <si>
-    <t>78970155027722432</t>
-  </si>
-  <si>
-    <t>78970155027722259</t>
-  </si>
-  <si>
-    <t>78970155027722374</t>
-  </si>
-  <si>
-    <t>78970155027722325</t>
-  </si>
-  <si>
-    <t>78970155027722333</t>
-  </si>
-  <si>
-    <t>78970155027722184</t>
+    <t>95 EKONOMY UNLEADED</t>
+  </si>
+  <si>
+    <t>DIESEL DOUBLE FILTER</t>
+  </si>
+  <si>
+    <t>E GAS LPG</t>
   </si>
   <si>
     <t>DIESEL EKONOMY</t>
   </si>
   <si>
-    <t>DIESEL DOUBLE FILTER</t>
-  </si>
-  <si>
-    <t>95 EKONOMY UNLEADED</t>
-  </si>
-  <si>
-    <t>E GAS LPG</t>
-  </si>
-  <si>
-    <t>11:21</t>
-  </si>
-  <si>
-    <t>15:42</t>
-  </si>
-  <si>
-    <t>10:38</t>
-  </si>
-  <si>
-    <t>12:33</t>
-  </si>
-  <si>
-    <t>16:36</t>
-  </si>
-  <si>
-    <t>17:10</t>
-  </si>
-  <si>
-    <t>18:51</t>
-  </si>
-  <si>
-    <t>09:46</t>
-  </si>
-  <si>
-    <t>14:27</t>
-  </si>
-  <si>
-    <t>08:49</t>
-  </si>
-  <si>
-    <t>12:30</t>
-  </si>
-  <si>
-    <t>17:32</t>
-  </si>
-  <si>
-    <t>11:42</t>
-  </si>
-  <si>
-    <t>13:11</t>
-  </si>
-  <si>
-    <t>12:49</t>
-  </si>
-  <si>
-    <t>13:24</t>
-  </si>
-  <si>
-    <t>14:18</t>
-  </si>
-  <si>
-    <t>16:05</t>
-  </si>
-  <si>
-    <t>12:26</t>
-  </si>
-  <si>
-    <t>17:17</t>
-  </si>
-  <si>
-    <t>08:38</t>
-  </si>
-  <si>
-    <t>09:32</t>
-  </si>
-  <si>
-    <t>12:56</t>
-  </si>
-  <si>
-    <t>19:01</t>
-  </si>
-  <si>
-    <t>08:10</t>
-  </si>
-  <si>
-    <t>12:20</t>
-  </si>
-  <si>
-    <t>14:25</t>
-  </si>
-  <si>
-    <t>15:14</t>
-  </si>
-  <si>
-    <t>16:17</t>
-  </si>
-  <si>
-    <t>11:24</t>
-  </si>
-  <si>
-    <t>13:34</t>
+    <t>10:57</t>
+  </si>
+  <si>
+    <t>11:50</t>
+  </si>
+  <si>
+    <t>14:05</t>
+  </si>
+  <si>
+    <t>12:14</t>
+  </si>
+  <si>
+    <t>14:14</t>
+  </si>
+  <si>
+    <t>14:55</t>
+  </si>
+  <si>
+    <t>13:42</t>
+  </si>
+  <si>
+    <t>10:09</t>
+  </si>
+  <si>
+    <t>11:25</t>
+  </si>
+  <si>
+    <t>14:17</t>
+  </si>
+  <si>
+    <t>16:02</t>
+  </si>
+  <si>
+    <t>11:15</t>
+  </si>
+  <si>
+    <t>11:20</t>
+  </si>
+  <si>
+    <t>14:50</t>
+  </si>
+  <si>
+    <t>07:56</t>
+  </si>
+  <si>
+    <t>12:59</t>
+  </si>
+  <si>
+    <t>17:05</t>
+  </si>
+  <si>
+    <t>10:53</t>
+  </si>
+  <si>
+    <t>14:22</t>
+  </si>
+  <si>
+    <t>11:17</t>
+  </si>
+  <si>
+    <t>13:01</t>
+  </si>
+  <si>
+    <t>14:34</t>
+  </si>
+  <si>
+    <t>15:34</t>
+  </si>
+  <si>
+    <t>10:11</t>
+  </si>
+  <si>
+    <t>17:33</t>
+  </si>
+  <si>
+    <t>14:36</t>
   </si>
   <si>
     <t>Общи литри по продукт / ОБЩИНА АКСАКОВО % 1</t>
@@ -725,7 +704,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M41"/>
+  <dimension ref="A1:M38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -789,40 +768,40 @@
         <v>13</v>
       </c>
       <c r="B2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C2" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D2" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E2" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F2">
-        <v>35.54</v>
+        <v>23.97</v>
       </c>
       <c r="G2" s="1">
-        <v>1.56</v>
+        <v>1.47</v>
       </c>
       <c r="H2">
-        <v>55.44</v>
+        <v>35.24</v>
       </c>
       <c r="I2" s="1">
-        <v>1.59</v>
+        <v>1.5</v>
       </c>
       <c r="J2">
-        <v>56.51</v>
+        <v>35.96</v>
       </c>
       <c r="K2" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L2">
-        <v>65992</v>
+        <v>0</v>
       </c>
       <c r="M2">
-        <v>115490</v>
+        <v>121086</v>
       </c>
     </row>
     <row r="3" spans="1:13">
@@ -830,81 +809,81 @@
         <v>13</v>
       </c>
       <c r="B3" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C3" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D3" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E3" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F3">
-        <v>67.17</v>
+        <v>67.54000000000001</v>
       </c>
       <c r="G3" s="1">
-        <v>1.85</v>
+        <v>1.77</v>
       </c>
       <c r="H3">
-        <v>124.26</v>
+        <v>119.55</v>
       </c>
       <c r="I3" s="1">
-        <v>1.85</v>
+        <v>1.77</v>
       </c>
       <c r="J3">
-        <v>124.26</v>
+        <v>119.55</v>
       </c>
       <c r="K3" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="L3">
         <v>0</v>
       </c>
       <c r="M3">
-        <v>200309</v>
+        <v>122136</v>
       </c>
     </row>
     <row r="4" spans="1:13">
       <c r="A4" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C4" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E4" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F4">
-        <v>42.77</v>
+        <v>29.5</v>
       </c>
       <c r="G4" s="1">
-        <v>1.52</v>
+        <v>0.65</v>
       </c>
       <c r="H4">
-        <v>65.01000000000001</v>
+        <v>19.18</v>
       </c>
       <c r="I4" s="1">
-        <v>1.55</v>
+        <v>0.66</v>
       </c>
       <c r="J4">
-        <v>66.29000000000001</v>
+        <v>19.47</v>
       </c>
       <c r="K4" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
       <c r="M4">
-        <v>115876</v>
+        <v>208968</v>
       </c>
     </row>
     <row r="5" spans="1:13">
@@ -912,40 +891,40 @@
         <v>14</v>
       </c>
       <c r="B5" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C5" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D5" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F5">
-        <v>70.38</v>
+        <v>44.2</v>
       </c>
       <c r="G5" s="1">
-        <v>1.56</v>
+        <v>1.48</v>
       </c>
       <c r="H5">
-        <v>109.79</v>
+        <v>65.42</v>
       </c>
       <c r="I5" s="1">
-        <v>1.59</v>
+        <v>1.51</v>
       </c>
       <c r="J5">
-        <v>111.9</v>
+        <v>66.73999999999999</v>
       </c>
       <c r="K5" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
       <c r="M5">
-        <v>115942</v>
+        <v>121528</v>
       </c>
     </row>
     <row r="6" spans="1:13">
@@ -953,40 +932,40 @@
         <v>14</v>
       </c>
       <c r="B6" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C6" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D6" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E6" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F6">
-        <v>29</v>
+        <v>26.49</v>
       </c>
       <c r="G6" s="1">
-        <v>1.52</v>
+        <v>1.48</v>
       </c>
       <c r="H6">
-        <v>44.08</v>
+        <v>39.21</v>
       </c>
       <c r="I6" s="1">
-        <v>1.55</v>
+        <v>1.51</v>
       </c>
       <c r="J6">
-        <v>44.95</v>
+        <v>40</v>
       </c>
       <c r="K6" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
       <c r="M6">
-        <v>200867</v>
+        <v>121593</v>
       </c>
     </row>
     <row r="7" spans="1:13">
@@ -994,163 +973,163 @@
         <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C7" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D7" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E7" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F7">
-        <v>25.31</v>
+        <v>31</v>
       </c>
       <c r="G7" s="1">
-        <v>0.66</v>
+        <v>1.47</v>
       </c>
       <c r="H7">
-        <v>16.7</v>
+        <v>45.57</v>
       </c>
       <c r="I7" s="1">
-        <v>0.67</v>
+        <v>1.5</v>
       </c>
       <c r="J7">
-        <v>16.96</v>
+        <v>46.5</v>
       </c>
       <c r="K7" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
       <c r="M7">
-        <v>116052</v>
+        <v>121634</v>
       </c>
     </row>
     <row r="8" spans="1:13">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B8" t="s">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="C8" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D8" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E8" t="s">
         <v>64</v>
       </c>
       <c r="F8">
-        <v>51.72</v>
+        <v>116</v>
       </c>
       <c r="G8" s="1">
-        <v>1.87</v>
+        <v>1.48</v>
       </c>
       <c r="H8">
-        <v>96.72</v>
+        <v>171.68</v>
       </c>
       <c r="I8" s="1">
-        <v>1.87</v>
+        <v>1.51</v>
       </c>
       <c r="J8">
-        <v>96.72</v>
+        <v>175.16</v>
       </c>
       <c r="K8" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
       <c r="M8">
-        <v>293557</v>
+        <v>122045</v>
       </c>
     </row>
     <row r="9" spans="1:13">
       <c r="A9" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B9" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C9" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D9" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E9" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F9">
-        <v>38.05</v>
+        <v>30</v>
       </c>
       <c r="G9" s="1">
-        <v>1.55</v>
+        <v>1.47</v>
       </c>
       <c r="H9">
-        <v>58.98</v>
+        <v>44.1</v>
       </c>
       <c r="I9" s="1">
-        <v>1.58</v>
+        <v>1.5</v>
       </c>
       <c r="J9">
-        <v>60.12</v>
+        <v>45</v>
       </c>
       <c r="K9" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L9">
         <v>0</v>
       </c>
       <c r="M9">
-        <v>116213</v>
+        <v>211614</v>
       </c>
     </row>
     <row r="10" spans="1:13">
       <c r="A10" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B10" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C10" t="s">
-        <v>36</v>
+        <v>28</v>
       </c>
       <c r="D10" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="E10" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="F10">
-        <v>32.31</v>
+        <v>61.29</v>
       </c>
       <c r="G10" s="1">
-        <v>1.52</v>
+        <v>1.78</v>
       </c>
       <c r="H10">
-        <v>49.11</v>
+        <v>109.1</v>
       </c>
       <c r="I10" s="1">
-        <v>1.55</v>
+        <v>1.78</v>
       </c>
       <c r="J10">
-        <v>50.08</v>
+        <v>109.1</v>
       </c>
       <c r="K10" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
       <c r="M10">
-        <v>201368</v>
+        <v>122989</v>
       </c>
     </row>
     <row r="11" spans="1:13">
@@ -1158,40 +1137,40 @@
         <v>16</v>
       </c>
       <c r="B11" t="s">
+        <v>24</v>
+      </c>
+      <c r="C11" t="s">
+        <v>35</v>
+      </c>
+      <c r="D11" t="s">
+        <v>52</v>
+      </c>
+      <c r="E11" t="s">
+        <v>64</v>
+      </c>
+      <c r="F11">
         <v>26</v>
       </c>
-      <c r="C11" t="s">
-        <v>37</v>
-      </c>
-      <c r="D11" t="s">
-        <v>54</v>
-      </c>
-      <c r="E11" t="s">
-        <v>63</v>
-      </c>
-      <c r="F11">
-        <v>48.06</v>
-      </c>
       <c r="G11" s="1">
-        <v>1.53</v>
+        <v>1.49</v>
       </c>
       <c r="H11">
-        <v>73.53</v>
+        <v>38.74</v>
       </c>
       <c r="I11" s="1">
-        <v>1.56</v>
+        <v>1.52</v>
       </c>
       <c r="J11">
-        <v>74.97</v>
+        <v>39.52</v>
       </c>
       <c r="K11" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="L11">
         <v>0</v>
       </c>
       <c r="M11">
-        <v>201756</v>
+        <v>211772</v>
       </c>
     </row>
     <row r="12" spans="1:13">
@@ -1199,40 +1178,40 @@
         <v>16</v>
       </c>
       <c r="B12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C12" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D12" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F12">
-        <v>122.01</v>
+        <v>56.22</v>
       </c>
       <c r="G12" s="1">
-        <v>1.53</v>
+        <v>1.49</v>
       </c>
       <c r="H12">
-        <v>186.68</v>
+        <v>83.77</v>
       </c>
       <c r="I12" s="1">
-        <v>1.56</v>
+        <v>1.52</v>
       </c>
       <c r="J12">
-        <v>190.34</v>
+        <v>85.45</v>
       </c>
       <c r="K12" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="L12">
         <v>0</v>
       </c>
       <c r="M12">
-        <v>201858</v>
+        <v>123104</v>
       </c>
     </row>
     <row r="13" spans="1:13">
@@ -1240,163 +1219,163 @@
         <v>17</v>
       </c>
       <c r="B13" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
       <c r="C13" t="s">
-        <v>30</v>
+        <v>37</v>
       </c>
       <c r="D13" t="s">
-        <v>47</v>
+        <v>54</v>
       </c>
       <c r="E13" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="F13">
-        <v>50</v>
+        <v>21.94</v>
       </c>
       <c r="G13" s="1">
-        <v>1.8</v>
+        <v>1.47</v>
       </c>
       <c r="H13">
-        <v>90</v>
+        <v>32.25</v>
       </c>
       <c r="I13" s="1">
-        <v>1.8</v>
+        <v>1.5</v>
       </c>
       <c r="J13">
-        <v>90</v>
+        <v>32.91</v>
       </c>
       <c r="K13" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
       <c r="M13">
-        <v>215010</v>
+        <v>212288</v>
       </c>
     </row>
     <row r="14" spans="1:13">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B14" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C14" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D14" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="E14" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F14">
-        <v>41.19</v>
+        <v>47.95</v>
       </c>
       <c r="G14" s="1">
-        <v>1.49</v>
+        <v>1.47</v>
       </c>
       <c r="H14">
-        <v>61.37</v>
+        <v>70.48999999999999</v>
       </c>
       <c r="I14" s="1">
-        <v>1.52</v>
+        <v>1.5</v>
       </c>
       <c r="J14">
-        <v>62.61</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="K14" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L14">
         <v>0</v>
       </c>
       <c r="M14">
-        <v>117752</v>
+        <v>212293</v>
       </c>
     </row>
     <row r="15" spans="1:13">
       <c r="A15" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C15" t="s">
-        <v>40</v>
+        <v>32</v>
       </c>
       <c r="D15" t="s">
-        <v>57</v>
+        <v>49</v>
       </c>
       <c r="E15" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F15">
-        <v>115.63</v>
+        <v>34</v>
       </c>
       <c r="G15" s="1">
-        <v>1.49</v>
+        <v>1.47</v>
       </c>
       <c r="H15">
-        <v>172.29</v>
+        <v>49.98</v>
       </c>
       <c r="I15" s="1">
-        <v>1.52</v>
+        <v>1.5</v>
       </c>
       <c r="J15">
-        <v>175.76</v>
+        <v>51</v>
       </c>
       <c r="K15" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="L15">
         <v>0</v>
       </c>
       <c r="M15">
-        <v>203469</v>
+        <v>123433</v>
       </c>
     </row>
     <row r="16" spans="1:13">
       <c r="A16" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C16" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D16" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E16" t="s">
-        <v>65</v>
+        <v>61</v>
       </c>
       <c r="F16">
-        <v>28.29</v>
+        <v>41.45</v>
       </c>
       <c r="G16" s="1">
-        <v>1.48</v>
+        <v>1.46</v>
       </c>
       <c r="H16">
-        <v>41.87</v>
+        <v>60.52</v>
       </c>
       <c r="I16" s="1">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="J16">
-        <v>42.72</v>
+        <v>61.76</v>
       </c>
       <c r="K16" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L16">
-        <v>85570</v>
+        <v>6068</v>
       </c>
       <c r="M16">
-        <v>204000</v>
+        <v>212689</v>
       </c>
     </row>
     <row r="17" spans="1:13">
@@ -1404,40 +1383,40 @@
         <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C17" t="s">
-        <v>42</v>
+        <v>33</v>
       </c>
       <c r="D17" t="s">
-        <v>59</v>
+        <v>50</v>
       </c>
       <c r="E17" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F17">
-        <v>42.06</v>
+        <v>146</v>
       </c>
       <c r="G17" s="1">
-        <v>1.48</v>
+        <v>1.49</v>
       </c>
       <c r="H17">
-        <v>62.25</v>
+        <v>217.54</v>
       </c>
       <c r="I17" s="1">
-        <v>1.51</v>
+        <v>1.52</v>
       </c>
       <c r="J17">
-        <v>63.51</v>
+        <v>221.92</v>
       </c>
       <c r="K17" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L17">
         <v>0</v>
       </c>
       <c r="M17">
-        <v>118213</v>
+        <v>124132</v>
       </c>
     </row>
     <row r="18" spans="1:13">
@@ -1445,81 +1424,81 @@
         <v>19</v>
       </c>
       <c r="B18" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C18" t="s">
-        <v>33</v>
+        <v>29</v>
       </c>
       <c r="D18" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="E18" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="F18">
-        <v>35</v>
+        <v>37.94</v>
       </c>
       <c r="G18" s="1">
-        <v>1.48</v>
+        <v>0.62</v>
       </c>
       <c r="H18">
-        <v>51.8</v>
+        <v>23.52</v>
       </c>
       <c r="I18" s="1">
-        <v>1.51</v>
+        <v>0.63</v>
       </c>
       <c r="J18">
-        <v>52.85</v>
+        <v>23.9</v>
       </c>
       <c r="K18" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L18">
-        <v>73832</v>
+        <v>0</v>
       </c>
       <c r="M18">
-        <v>204054</v>
+        <v>124232</v>
       </c>
     </row>
     <row r="19" spans="1:13">
       <c r="A19" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B19" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
       <c r="D19" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E19" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F19">
-        <v>56.9</v>
+        <v>32.35</v>
       </c>
       <c r="G19" s="1">
-        <v>1.49</v>
+        <v>1.51</v>
       </c>
       <c r="H19">
-        <v>84.78</v>
+        <v>48.85</v>
       </c>
       <c r="I19" s="1">
-        <v>1.52</v>
+        <v>1.54</v>
       </c>
       <c r="J19">
-        <v>86.48999999999999</v>
+        <v>49.82</v>
       </c>
       <c r="K19" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L19">
         <v>0</v>
       </c>
       <c r="M19">
-        <v>118260</v>
+        <v>213994</v>
       </c>
     </row>
     <row r="20" spans="1:13">
@@ -1527,81 +1506,81 @@
         <v>20</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C20" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="D20" t="s">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="E20" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F20">
-        <v>138</v>
+        <v>31</v>
       </c>
       <c r="G20" s="1">
-        <v>1.48</v>
+        <v>1.46</v>
       </c>
       <c r="H20">
-        <v>204.24</v>
+        <v>45.26</v>
       </c>
       <c r="I20" s="1">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="J20">
-        <v>208.38</v>
+        <v>46.19</v>
       </c>
       <c r="K20" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L20">
         <v>0</v>
       </c>
       <c r="M20">
-        <v>204494</v>
+        <v>124636</v>
       </c>
     </row>
     <row r="21" spans="1:13">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B21" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C21" t="s">
-        <v>34</v>
+        <v>41</v>
       </c>
       <c r="D21" t="s">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="E21" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="F21">
-        <v>31.91</v>
+        <v>18.03</v>
       </c>
       <c r="G21" s="1">
-        <v>0.65</v>
+        <v>1.46</v>
       </c>
       <c r="H21">
-        <v>20.74</v>
+        <v>26.32</v>
       </c>
       <c r="I21" s="1">
-        <v>0.66</v>
+        <v>1.49</v>
       </c>
       <c r="J21">
-        <v>21.06</v>
+        <v>26.86</v>
       </c>
       <c r="K21" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="L21">
         <v>0</v>
       </c>
       <c r="M21">
-        <v>118717</v>
+        <v>215932</v>
       </c>
     </row>
     <row r="22" spans="1:13">
@@ -1609,40 +1588,40 @@
         <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C22" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="D22" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="E22" t="s">
         <v>64</v>
       </c>
       <c r="F22">
-        <v>59.57</v>
+        <v>143</v>
       </c>
       <c r="G22" s="1">
-        <v>1.77</v>
+        <v>1.53</v>
       </c>
       <c r="H22">
-        <v>105.44</v>
+        <v>218.79</v>
       </c>
       <c r="I22" s="1">
-        <v>1.77</v>
+        <v>1.56</v>
       </c>
       <c r="J22">
-        <v>105.44</v>
+        <v>223.08</v>
       </c>
       <c r="K22" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L22">
         <v>0</v>
       </c>
       <c r="M22">
-        <v>204980</v>
+        <v>216006</v>
       </c>
     </row>
     <row r="23" spans="1:13">
@@ -1650,81 +1629,81 @@
         <v>21</v>
       </c>
       <c r="B23" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C23" t="s">
-        <v>44</v>
+        <v>31</v>
       </c>
       <c r="D23" t="s">
-        <v>61</v>
+        <v>48</v>
       </c>
       <c r="E23" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F23">
-        <v>28.16</v>
+        <v>33.84</v>
       </c>
       <c r="G23" s="1">
-        <v>1.48</v>
+        <v>1.53</v>
       </c>
       <c r="H23">
-        <v>41.68</v>
+        <v>51.78</v>
       </c>
       <c r="I23" s="1">
-        <v>1.51</v>
+        <v>1.56</v>
       </c>
       <c r="J23">
-        <v>42.52</v>
+        <v>52.79</v>
       </c>
       <c r="K23" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="L23">
         <v>0</v>
       </c>
       <c r="M23">
-        <v>205046</v>
+        <v>216086</v>
       </c>
     </row>
     <row r="24" spans="1:13">
       <c r="A24" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B24" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C24" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D24" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E24" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F24">
-        <v>107</v>
+        <v>39.46</v>
       </c>
       <c r="G24" s="1">
-        <v>1.48</v>
+        <v>1.46</v>
       </c>
       <c r="H24">
-        <v>158.36</v>
+        <v>57.61</v>
       </c>
       <c r="I24" s="1">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="J24">
-        <v>161.57</v>
+        <v>58.8</v>
       </c>
       <c r="K24" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="L24">
-        <v>0</v>
+        <v>118440</v>
       </c>
       <c r="M24">
-        <v>119188</v>
+        <v>216115</v>
       </c>
     </row>
     <row r="25" spans="1:13">
@@ -1732,122 +1711,122 @@
         <v>22</v>
       </c>
       <c r="B25" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C25" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D25" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E25" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F25">
-        <v>31.49</v>
+        <v>23</v>
       </c>
       <c r="G25" s="1">
-        <v>1.48</v>
+        <v>1.46</v>
       </c>
       <c r="H25">
-        <v>46.61</v>
+        <v>33.58</v>
       </c>
       <c r="I25" s="1">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="J25">
-        <v>47.55</v>
+        <v>34.27</v>
       </c>
       <c r="K25" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="L25">
         <v>0</v>
       </c>
       <c r="M25">
-        <v>206084</v>
+        <v>216507</v>
       </c>
     </row>
     <row r="26" spans="1:13">
       <c r="A26" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B26" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C26" t="s">
-        <v>32</v>
+        <v>43</v>
       </c>
       <c r="D26" t="s">
-        <v>49</v>
+        <v>60</v>
       </c>
       <c r="E26" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F26">
-        <v>66.48999999999999</v>
+        <v>40.82</v>
       </c>
       <c r="G26" s="1">
-        <v>1.48</v>
+        <v>1.46</v>
       </c>
       <c r="H26">
-        <v>98.41</v>
+        <v>59.6</v>
       </c>
       <c r="I26" s="1">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="J26">
-        <v>100.4</v>
+        <v>60.82</v>
       </c>
       <c r="K26" t="s">
-        <v>91</v>
+        <v>70</v>
       </c>
       <c r="L26">
         <v>0</v>
       </c>
       <c r="M26">
-        <v>207379</v>
+        <v>216702</v>
       </c>
     </row>
     <row r="27" spans="1:13">
       <c r="A27" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B27" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C27" t="s">
-        <v>38</v>
+        <v>30</v>
       </c>
       <c r="D27" t="s">
-        <v>55</v>
+        <v>47</v>
       </c>
       <c r="E27" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="F27">
-        <v>132.01</v>
+        <v>64.29000000000001</v>
       </c>
       <c r="G27" s="1">
-        <v>1.48</v>
+        <v>1.53</v>
       </c>
       <c r="H27">
-        <v>195.37</v>
+        <v>98.36</v>
       </c>
       <c r="I27" s="1">
-        <v>1.51</v>
+        <v>1.56</v>
       </c>
       <c r="J27">
-        <v>199.34</v>
+        <v>100.29</v>
       </c>
       <c r="K27" t="s">
-        <v>92</v>
+        <v>89</v>
       </c>
       <c r="L27">
         <v>0</v>
       </c>
       <c r="M27">
-        <v>120372</v>
+        <v>216786</v>
       </c>
     </row>
     <row r="28" spans="1:13">
@@ -1855,40 +1834,40 @@
         <v>23</v>
       </c>
       <c r="B28" t="s">
+        <v>24</v>
+      </c>
+      <c r="C28" t="s">
+        <v>32</v>
+      </c>
+      <c r="D28" t="s">
+        <v>49</v>
+      </c>
+      <c r="E28" t="s">
+        <v>61</v>
+      </c>
+      <c r="F28">
         <v>26</v>
       </c>
-      <c r="C28" t="s">
-        <v>35</v>
-      </c>
-      <c r="D28" t="s">
-        <v>52</v>
-      </c>
-      <c r="E28" t="s">
-        <v>63</v>
-      </c>
-      <c r="F28">
-        <v>33.8</v>
-      </c>
       <c r="G28" s="1">
-        <v>1.48</v>
+        <v>1.46</v>
       </c>
       <c r="H28">
-        <v>50.02</v>
+        <v>37.96</v>
       </c>
       <c r="I28" s="1">
-        <v>1.51</v>
+        <v>1.49</v>
       </c>
       <c r="J28">
-        <v>51.04</v>
+        <v>38.74</v>
       </c>
       <c r="K28" t="s">
-        <v>93</v>
+        <v>83</v>
       </c>
       <c r="L28">
         <v>0</v>
       </c>
       <c r="M28">
-        <v>120440</v>
+        <v>126388</v>
       </c>
     </row>
     <row r="29" spans="1:13">
@@ -1896,193 +1875,130 @@
         <v>23</v>
       </c>
       <c r="B29" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="C29" t="s">
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="D29" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="E29" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="F29">
-        <v>35.99</v>
+        <v>61.95</v>
       </c>
       <c r="G29" s="1">
-        <v>1.47</v>
+        <v>1.55</v>
       </c>
       <c r="H29">
-        <v>52.91</v>
+        <v>96.02</v>
       </c>
       <c r="I29" s="1">
-        <v>1.5</v>
+        <v>1.58</v>
       </c>
       <c r="J29">
-        <v>53.98</v>
+        <v>97.88</v>
       </c>
       <c r="K29" t="s">
+        <v>90</v>
+      </c>
+      <c r="L29">
+        <v>0</v>
+      </c>
+      <c r="M29">
+        <v>126397</v>
+      </c>
+    </row>
+    <row r="32" spans="1:13">
+      <c r="A32" s="3" t="s">
+        <v>91</v>
+      </c>
+      <c r="B32" s="3"/>
+      <c r="C32" s="3"/>
+      <c r="D32" s="3"/>
+      <c r="E32" s="3"/>
+      <c r="F32" s="3"/>
+    </row>
+    <row r="33" spans="1:6">
+      <c r="A33" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="B33" s="4" t="s">
+        <v>93</v>
+      </c>
+      <c r="C33" s="4" t="s">
         <v>94</v>
       </c>
-      <c r="L29">
-        <v>0</v>
-      </c>
-      <c r="M29">
-        <v>207651</v>
-      </c>
-    </row>
-    <row r="30" spans="1:13">
-      <c r="A30" t="s">
-        <v>23</v>
-      </c>
-      <c r="B30" t="s">
-        <v>26</v>
-      </c>
-      <c r="C30" t="s">
-        <v>42</v>
-      </c>
-      <c r="D30" t="s">
-        <v>59</v>
-      </c>
-      <c r="E30" t="s">
-        <v>65</v>
-      </c>
-      <c r="F30">
-        <v>44.92</v>
-      </c>
-      <c r="G30" s="1">
-        <v>1.47</v>
-      </c>
-      <c r="H30">
-        <v>66.03</v>
-      </c>
-      <c r="I30" s="1">
-        <v>1.5</v>
-      </c>
-      <c r="J30">
-        <v>67.38</v>
-      </c>
-      <c r="K30" t="s">
+      <c r="D33" s="4" t="s">
         <v>95</v>
       </c>
-      <c r="L30">
-        <v>0</v>
-      </c>
-      <c r="M30">
-        <v>120506</v>
-      </c>
-    </row>
-    <row r="31" spans="1:13">
-      <c r="A31" t="s">
-        <v>24</v>
-      </c>
-      <c r="B31" t="s">
-        <v>26</v>
-      </c>
-      <c r="C31" t="s">
-        <v>36</v>
-      </c>
-      <c r="D31" t="s">
-        <v>53</v>
-      </c>
-      <c r="E31" t="s">
-        <v>65</v>
-      </c>
-      <c r="F31">
-        <v>30.69</v>
-      </c>
-      <c r="G31" s="1">
-        <v>1.47</v>
-      </c>
-      <c r="H31">
-        <v>45.11</v>
-      </c>
-      <c r="I31" s="1">
-        <v>1.5</v>
-      </c>
-      <c r="J31">
-        <v>46.04</v>
-      </c>
-      <c r="K31" t="s">
-        <v>96</v>
-      </c>
-      <c r="L31">
-        <v>0</v>
-      </c>
-      <c r="M31">
-        <v>208152</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13">
-      <c r="A32" t="s">
-        <v>24</v>
-      </c>
-      <c r="B32" t="s">
-        <v>26</v>
-      </c>
-      <c r="C32" t="s">
-        <v>39</v>
-      </c>
-      <c r="D32" t="s">
-        <v>56</v>
-      </c>
-      <c r="E32" t="s">
-        <v>63</v>
-      </c>
-      <c r="F32">
-        <v>34.64</v>
-      </c>
-      <c r="G32" s="1">
-        <v>1.48</v>
-      </c>
-      <c r="H32">
-        <v>51.27</v>
-      </c>
-      <c r="I32" s="1">
-        <v>1.51</v>
-      </c>
-      <c r="J32">
-        <v>52.31</v>
-      </c>
-      <c r="K32" t="s">
-        <v>97</v>
-      </c>
-      <c r="L32">
-        <v>0</v>
-      </c>
-      <c r="M32">
-        <v>208237</v>
+      <c r="E33" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="F33" s="4" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6">
+      <c r="A34" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="B34" s="6">
+        <v>750.34</v>
+      </c>
+      <c r="C34" s="6">
+        <v>11</v>
+      </c>
+      <c r="D34" s="7">
+        <v>1.5062</v>
+      </c>
+      <c r="E34" s="6">
+        <v>1130.16</v>
+      </c>
+      <c r="F34" s="6">
+        <v>1152.65</v>
       </c>
     </row>
     <row r="35" spans="1:6">
-      <c r="A35" s="3" t="s">
-        <v>98</v>
-      </c>
-      <c r="B35" s="3"/>
-      <c r="C35" s="3"/>
-      <c r="D35" s="3"/>
-      <c r="E35" s="3"/>
-      <c r="F35" s="3"/>
+      <c r="A35" s="5" t="s">
+        <v>61</v>
+      </c>
+      <c r="B35" s="6">
+        <v>408.62</v>
+      </c>
+      <c r="C35" s="6">
+        <v>13</v>
+      </c>
+      <c r="D35" s="7">
+        <v>1.4646</v>
+      </c>
+      <c r="E35" s="6">
+        <v>598.48</v>
+      </c>
+      <c r="F35" s="6">
+        <v>610.74</v>
+      </c>
     </row>
     <row r="36" spans="1:6">
-      <c r="A36" s="4" t="s">
-        <v>99</v>
-      </c>
-      <c r="B36" s="4" t="s">
-        <v>100</v>
-      </c>
-      <c r="C36" s="4" t="s">
-        <v>101</v>
-      </c>
-      <c r="D36" s="4" t="s">
-        <v>102</v>
-      </c>
-      <c r="E36" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="F36" s="4" t="s">
-        <v>9</v>
+      <c r="A36" s="5" t="s">
+        <v>62</v>
+      </c>
+      <c r="B36" s="6">
+        <v>128.83</v>
+      </c>
+      <c r="C36" s="6">
+        <v>2</v>
+      </c>
+      <c r="D36" s="7">
+        <v>1.7748</v>
+      </c>
+      <c r="E36" s="6">
+        <v>228.65</v>
+      </c>
+      <c r="F36" s="6">
+        <v>228.65</v>
       </c>
     </row>
     <row r="37" spans="1:6">
@@ -2090,102 +2006,42 @@
         <v>63</v>
       </c>
       <c r="B37" s="6">
-        <v>1071.19</v>
+        <v>67.44</v>
       </c>
       <c r="C37" s="6">
-        <v>15</v>
+        <v>2</v>
       </c>
       <c r="D37" s="7">
-        <v>1.5003</v>
+        <v>0.6332</v>
       </c>
       <c r="E37" s="6">
-        <v>1607.14</v>
+        <v>42.7</v>
       </c>
       <c r="F37" s="6">
-        <v>1639.29</v>
+        <v>43.37</v>
       </c>
     </row>
     <row r="38" spans="1:6">
-      <c r="A38" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="B38" s="6">
-        <v>349.19</v>
-      </c>
-      <c r="C38" s="6">
-        <v>10</v>
-      </c>
-      <c r="D38" s="7">
-        <v>1.4887</v>
-      </c>
-      <c r="E38" s="6">
-        <v>519.85</v>
-      </c>
-      <c r="F38" s="6">
-        <v>530.3200000000001</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6">
-      <c r="A39" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="B39" s="6">
-        <v>228.46</v>
-      </c>
-      <c r="C39" s="6">
-        <v>4</v>
-      </c>
-      <c r="D39" s="7">
-        <v>1.8227</v>
-      </c>
-      <c r="E39" s="6">
-        <v>416.42</v>
-      </c>
-      <c r="F39" s="6">
-        <v>416.42</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6">
-      <c r="A40" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="B40" s="6">
-        <v>57.22</v>
-      </c>
-      <c r="C40" s="6">
-        <v>2</v>
-      </c>
-      <c r="D40" s="7">
-        <v>0.6543</v>
-      </c>
-      <c r="E40" s="6">
-        <v>37.44</v>
-      </c>
-      <c r="F40" s="6">
-        <v>38.02</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6">
-      <c r="A41" s="8" t="s">
-        <v>103</v>
-      </c>
-      <c r="B41" s="9">
-        <v>1706.06</v>
-      </c>
-      <c r="C41" s="9">
-        <v>31</v>
-      </c>
-      <c r="D41" s="7"/>
-      <c r="E41" s="9">
-        <v>2580.85</v>
-      </c>
-      <c r="F41" s="9">
-        <v>2624.05</v>
+      <c r="A38" s="8" t="s">
+        <v>96</v>
+      </c>
+      <c r="B38" s="9">
+        <v>1355.23</v>
+      </c>
+      <c r="C38" s="9">
+        <v>28</v>
+      </c>
+      <c r="D38" s="7"/>
+      <c r="E38" s="9">
+        <v>1999.99</v>
+      </c>
+      <c r="F38" s="9">
+        <v>2035.41</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A35:F35"/>
+    <mergeCell ref="A32:F32"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
ADD: final update - 01-15.07.2026 invoice files
</commit_message>
<xml_diff>
--- a/SPLIT_COMPANY_DATA/RESULT/companies_result/ОБЩИНА АКСАКОВО % 1/ОБЩИНА АКСАКОВО % 1.xlsx
+++ b/SPLIT_COMPANY_DATA/RESULT/companies_result/ОБЩИНА АКСАКОВО % 1/ОБЩИНА АКСАКОВО % 1.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="204" uniqueCount="97">
   <si>
     <t>Дата</t>
   </si>
@@ -52,9 +52,6 @@
     <t>Километри</t>
   </si>
   <si>
-    <t>Billing_Document</t>
-  </si>
-  <si>
     <t>2026-07-01</t>
   </si>
   <si>
@@ -88,13 +85,10 @@
     <t>2026-07-15</t>
   </si>
   <si>
-    <t>1147 Варна Ситроен</t>
-  </si>
-  <si>
-    <t>1158 Варна Чайка</t>
-  </si>
-  <si>
-    <t>1146 Варна Сливница</t>
+    <t>Варна Варненчик</t>
+  </si>
+  <si>
+    <t>Варна Чайка</t>
   </si>
   <si>
     <t>В2278РВ</t>
@@ -202,7 +196,7 @@
     <t>95 EKONOMY UNLEADED</t>
   </si>
   <si>
-    <t>DIESEL DOUBLE FILTER</t>
+    <t>DIESEL DOUBLE FILTERED</t>
   </si>
   <si>
     <t>E GAS LPG</t>
@@ -211,82 +205,88 @@
     <t>DIESEL EKONOMY</t>
   </si>
   <si>
-    <t>10:57</t>
-  </si>
-  <si>
-    <t>11:50</t>
-  </si>
-  <si>
-    <t>14:05</t>
-  </si>
-  <si>
-    <t>12:14</t>
-  </si>
-  <si>
-    <t>14:14</t>
-  </si>
-  <si>
-    <t>14:55</t>
-  </si>
-  <si>
-    <t>13:42</t>
-  </si>
-  <si>
-    <t>10:09</t>
-  </si>
-  <si>
-    <t>11:25</t>
-  </si>
-  <si>
-    <t>14:17</t>
-  </si>
-  <si>
-    <t>16:02</t>
-  </si>
-  <si>
-    <t>11:15</t>
-  </si>
-  <si>
-    <t>11:20</t>
-  </si>
-  <si>
-    <t>14:50</t>
-  </si>
-  <si>
-    <t>07:56</t>
-  </si>
-  <si>
-    <t>12:59</t>
-  </si>
-  <si>
-    <t>17:05</t>
-  </si>
-  <si>
-    <t>10:53</t>
-  </si>
-  <si>
-    <t>14:22</t>
-  </si>
-  <si>
-    <t>11:17</t>
-  </si>
-  <si>
-    <t>13:01</t>
-  </si>
-  <si>
-    <t>14:34</t>
-  </si>
-  <si>
-    <t>15:34</t>
-  </si>
-  <si>
-    <t>10:11</t>
-  </si>
-  <si>
-    <t>17:33</t>
-  </si>
-  <si>
-    <t>14:36</t>
+    <t>2026-07-01 10:57:07</t>
+  </si>
+  <si>
+    <t>2026-07-01 11:50:56</t>
+  </si>
+  <si>
+    <t>2026-07-01 14:05:38</t>
+  </si>
+  <si>
+    <t>2026-07-02 12:14:55</t>
+  </si>
+  <si>
+    <t>2026-07-02 14:14:38</t>
+  </si>
+  <si>
+    <t>2026-07-02 14:55:24</t>
+  </si>
+  <si>
+    <t>2026-07-03 13:42:32</t>
+  </si>
+  <si>
+    <t>2026-07-06 10:09:03</t>
+  </si>
+  <si>
+    <t>2026-07-06 11:25:37</t>
+  </si>
+  <si>
+    <t>2026-07-06 14:17:15</t>
+  </si>
+  <si>
+    <t>2026-07-06 16:02:57</t>
+  </si>
+  <si>
+    <t>2026-07-07 11:15:46</t>
+  </si>
+  <si>
+    <t>2026-07-07 11:20:17</t>
+  </si>
+  <si>
+    <t>2026-07-07 14:50:27</t>
+  </si>
+  <si>
+    <t>2026-07-08 07:56:09</t>
+  </si>
+  <si>
+    <t>2026-07-09 12:59:12</t>
+  </si>
+  <si>
+    <t>2026-07-09 17:05:51</t>
+  </si>
+  <si>
+    <t>2026-07-10 10:53:34</t>
+  </si>
+  <si>
+    <t>2026-07-10 14:22:06</t>
+  </si>
+  <si>
+    <t>2026-07-13 11:17:08</t>
+  </si>
+  <si>
+    <t>2026-07-13 13:01:54</t>
+  </si>
+  <si>
+    <t>2026-07-13 14:34:56</t>
+  </si>
+  <si>
+    <t>2026-07-13 15:34:19</t>
+  </si>
+  <si>
+    <t>2026-07-14 10:11:34</t>
+  </si>
+  <si>
+    <t>2026-07-14 14:55:01</t>
+  </si>
+  <si>
+    <t>2026-07-14 17:33:22</t>
+  </si>
+  <si>
+    <t>2026-07-15 14:22:35</t>
+  </si>
+  <si>
+    <t>2026-07-15 14:36:06</t>
   </si>
   <si>
     <t>Общи литри по продукт / ОБЩИНА АКСАКОВО % 1</t>
@@ -704,7 +704,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:M38"/>
+  <dimension ref="A1:L38"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="35.7109375" customWidth="1"/>
@@ -717,12 +717,11 @@
     <col min="8" max="8" width="23.7109375" customWidth="1"/>
     <col min="9" max="9" width="15.7109375" style="1" customWidth="1"/>
     <col min="10" max="10" width="23.7109375" customWidth="1"/>
-    <col min="11" max="11" width="7.7109375" customWidth="1"/>
+    <col min="11" max="11" width="21.7109375" customWidth="1"/>
     <col min="12" max="12" width="11.7109375" customWidth="1"/>
-    <col min="13" max="13" width="18.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13">
+    <row r="1" spans="1:12">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -759,25 +758,22 @@
       <c r="L1" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="2" t="s">
+    </row>
+    <row r="2" spans="1:12">
+      <c r="A2" t="s">
         <v>12</v>
       </c>
-    </row>
-    <row r="2" spans="1:13">
-      <c r="A2" t="s">
-        <v>13</v>
-      </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D2" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="E2" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F2">
         <v>23.97</v>
@@ -795,39 +791,36 @@
         <v>35.96</v>
       </c>
       <c r="K2" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="L2">
         <v>0</v>
       </c>
-      <c r="M2">
-        <v>121086</v>
-      </c>
-    </row>
-    <row r="3" spans="1:13">
+    </row>
+    <row r="3" spans="1:12">
       <c r="A3" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C3" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D3" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E3" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F3">
         <v>67.54000000000001</v>
       </c>
       <c r="G3" s="1">
-        <v>1.77</v>
+        <v>1.74</v>
       </c>
       <c r="H3">
-        <v>119.55</v>
+        <v>117.52</v>
       </c>
       <c r="I3" s="1">
         <v>1.77</v>
@@ -836,30 +829,27 @@
         <v>119.55</v>
       </c>
       <c r="K3" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="L3">
         <v>0</v>
       </c>
-      <c r="M3">
-        <v>122136</v>
-      </c>
-    </row>
-    <row r="4" spans="1:13">
+    </row>
+    <row r="4" spans="1:12">
       <c r="A4" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="B4" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D4" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E4" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F4">
         <v>29.5</v>
@@ -877,30 +867,27 @@
         <v>19.47</v>
       </c>
       <c r="K4" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="L4">
         <v>0</v>
       </c>
-      <c r="M4">
-        <v>208968</v>
-      </c>
-    </row>
-    <row r="5" spans="1:13">
+    </row>
+    <row r="5" spans="1:12">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B5" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F5">
         <v>44.2</v>
@@ -918,30 +905,27 @@
         <v>66.73999999999999</v>
       </c>
       <c r="K5" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="L5">
         <v>0</v>
       </c>
-      <c r="M5">
-        <v>121528</v>
-      </c>
-    </row>
-    <row r="6" spans="1:13">
+    </row>
+    <row r="6" spans="1:12">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B6" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C6" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D6" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E6" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F6">
         <v>26.49</v>
@@ -959,30 +943,27 @@
         <v>40</v>
       </c>
       <c r="K6" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="L6">
         <v>0</v>
       </c>
-      <c r="M6">
-        <v>121593</v>
-      </c>
-    </row>
-    <row r="7" spans="1:13">
+    </row>
+    <row r="7" spans="1:12">
       <c r="A7" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B7" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C7" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D7" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E7" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F7">
         <v>31</v>
@@ -1000,30 +981,27 @@
         <v>46.5</v>
       </c>
       <c r="K7" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="L7">
         <v>0</v>
       </c>
-      <c r="M7">
-        <v>121634</v>
-      </c>
-    </row>
-    <row r="8" spans="1:13">
+    </row>
+    <row r="8" spans="1:12">
       <c r="A8" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B8" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C8" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D8" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E8" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F8">
         <v>116</v>
@@ -1041,30 +1019,27 @@
         <v>175.16</v>
       </c>
       <c r="K8" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="L8">
         <v>0</v>
       </c>
-      <c r="M8">
-        <v>122045</v>
-      </c>
-    </row>
-    <row r="9" spans="1:13">
+    </row>
+    <row r="9" spans="1:12">
       <c r="A9" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B9" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C9" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="D9" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E9" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F9">
         <v>30</v>
@@ -1082,39 +1057,36 @@
         <v>45</v>
       </c>
       <c r="K9" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="L9">
         <v>0</v>
       </c>
-      <c r="M9">
-        <v>211614</v>
-      </c>
-    </row>
-    <row r="10" spans="1:13">
+    </row>
+    <row r="10" spans="1:12">
       <c r="A10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B10" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C10" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="D10" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E10" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="F10">
         <v>61.29</v>
       </c>
       <c r="G10" s="1">
-        <v>1.78</v>
+        <v>1.75</v>
       </c>
       <c r="H10">
-        <v>109.1</v>
+        <v>107.26</v>
       </c>
       <c r="I10" s="1">
         <v>1.78</v>
@@ -1123,30 +1095,27 @@
         <v>109.1</v>
       </c>
       <c r="K10" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="L10">
         <v>0</v>
       </c>
-      <c r="M10">
-        <v>122989</v>
-      </c>
-    </row>
-    <row r="11" spans="1:13">
+    </row>
+    <row r="11" spans="1:12">
       <c r="A11" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B11" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="D11" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="E11" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F11">
         <v>26</v>
@@ -1164,30 +1133,27 @@
         <v>39.52</v>
       </c>
       <c r="K11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="L11">
         <v>0</v>
       </c>
-      <c r="M11">
-        <v>211772</v>
-      </c>
-    </row>
-    <row r="12" spans="1:13">
+    </row>
+    <row r="12" spans="1:12">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="B12" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C12" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D12" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E12" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F12">
         <v>56.22</v>
@@ -1205,30 +1171,27 @@
         <v>85.45</v>
       </c>
       <c r="K12" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="L12">
         <v>0</v>
       </c>
-      <c r="M12">
-        <v>123104</v>
-      </c>
-    </row>
-    <row r="13" spans="1:13">
+    </row>
+    <row r="13" spans="1:12">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B13" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C13" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="D13" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E13" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F13">
         <v>21.94</v>
@@ -1246,30 +1209,27 @@
         <v>32.91</v>
       </c>
       <c r="K13" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="L13">
         <v>0</v>
       </c>
-      <c r="M13">
-        <v>212288</v>
-      </c>
-    </row>
-    <row r="14" spans="1:13">
+    </row>
+    <row r="14" spans="1:12">
       <c r="A14" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C14" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D14" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E14" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F14">
         <v>47.95</v>
@@ -1287,30 +1247,27 @@
         <v>71.93000000000001</v>
       </c>
       <c r="K14" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="L14">
         <v>0</v>
       </c>
-      <c r="M14">
-        <v>212293</v>
-      </c>
-    </row>
-    <row r="15" spans="1:13">
+    </row>
+    <row r="15" spans="1:12">
       <c r="A15" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="B15" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D15" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E15" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F15">
         <v>34</v>
@@ -1328,30 +1285,27 @@
         <v>51</v>
       </c>
       <c r="K15" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="L15">
         <v>0</v>
       </c>
-      <c r="M15">
-        <v>123433</v>
-      </c>
-    </row>
-    <row r="16" spans="1:13">
+    </row>
+    <row r="16" spans="1:12">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="B16" t="s">
-        <v>26</v>
+        <v>23</v>
       </c>
       <c r="C16" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="D16" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="E16" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F16">
         <v>41.45</v>
@@ -1369,30 +1323,27 @@
         <v>61.76</v>
       </c>
       <c r="K16" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="L16">
-        <v>6068</v>
-      </c>
-      <c r="M16">
-        <v>212689</v>
-      </c>
-    </row>
-    <row r="17" spans="1:13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:12">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B17" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C17" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D17" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E17" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F17">
         <v>146</v>
@@ -1410,30 +1361,27 @@
         <v>221.92</v>
       </c>
       <c r="K17" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="L17">
         <v>0</v>
       </c>
-      <c r="M17">
-        <v>124132</v>
-      </c>
-    </row>
-    <row r="18" spans="1:13">
+    </row>
+    <row r="18" spans="1:12">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D18" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="E18" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F18">
         <v>37.94</v>
@@ -1451,30 +1399,27 @@
         <v>23.9</v>
       </c>
       <c r="K18" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
       <c r="L18">
         <v>0</v>
       </c>
-      <c r="M18">
-        <v>124232</v>
-      </c>
-    </row>
-    <row r="19" spans="1:13">
+    </row>
+    <row r="19" spans="1:12">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B19" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="E19" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F19">
         <v>32.35</v>
@@ -1492,30 +1437,27 @@
         <v>49.82</v>
       </c>
       <c r="K19" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="L19">
         <v>0</v>
       </c>
-      <c r="M19">
-        <v>213994</v>
-      </c>
-    </row>
-    <row r="20" spans="1:13">
+    </row>
+    <row r="20" spans="1:12">
       <c r="A20" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C20" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D20" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E20" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F20">
         <v>31</v>
@@ -1533,30 +1475,27 @@
         <v>46.19</v>
       </c>
       <c r="K20" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="L20">
         <v>0</v>
       </c>
-      <c r="M20">
-        <v>124636</v>
-      </c>
-    </row>
-    <row r="21" spans="1:13">
+    </row>
+    <row r="21" spans="1:12">
       <c r="A21" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B21" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C21" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="D21" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="E21" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F21">
         <v>18.03</v>
@@ -1574,30 +1513,27 @@
         <v>26.86</v>
       </c>
       <c r="K21" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="L21">
         <v>0</v>
       </c>
-      <c r="M21">
-        <v>215932</v>
-      </c>
-    </row>
-    <row r="22" spans="1:13">
+    </row>
+    <row r="22" spans="1:12">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B22" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C22" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D22" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="E22" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F22">
         <v>143</v>
@@ -1615,30 +1551,27 @@
         <v>223.08</v>
       </c>
       <c r="K22" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="L22">
         <v>0</v>
       </c>
-      <c r="M22">
-        <v>216006</v>
-      </c>
-    </row>
-    <row r="23" spans="1:13">
+    </row>
+    <row r="23" spans="1:12">
       <c r="A23" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B23" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C23" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D23" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E23" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F23">
         <v>33.84</v>
@@ -1656,30 +1589,27 @@
         <v>52.79</v>
       </c>
       <c r="K23" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="L23">
         <v>0</v>
       </c>
-      <c r="M23">
-        <v>216086</v>
-      </c>
-    </row>
-    <row r="24" spans="1:13">
+    </row>
+    <row r="24" spans="1:12">
       <c r="A24" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B24" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C24" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D24" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="E24" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F24">
         <v>39.46</v>
@@ -1697,30 +1627,27 @@
         <v>58.8</v>
       </c>
       <c r="K24" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="L24">
-        <v>118440</v>
-      </c>
-      <c r="M24">
-        <v>216115</v>
-      </c>
-    </row>
-    <row r="25" spans="1:13">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:12">
       <c r="A25" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B25" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C25" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D25" t="s">
+        <v>57</v>
+      </c>
+      <c r="E25" t="s">
         <v>59</v>
-      </c>
-      <c r="E25" t="s">
-        <v>61</v>
       </c>
       <c r="F25">
         <v>23</v>
@@ -1738,30 +1665,27 @@
         <v>34.27</v>
       </c>
       <c r="K25" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="L25">
         <v>0</v>
       </c>
-      <c r="M25">
-        <v>216507</v>
-      </c>
-    </row>
-    <row r="26" spans="1:13">
+    </row>
+    <row r="26" spans="1:12">
       <c r="A26" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B26" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C26" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="D26" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E26" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F26">
         <v>40.82</v>
@@ -1779,30 +1703,27 @@
         <v>60.82</v>
       </c>
       <c r="K26" t="s">
-        <v>70</v>
+        <v>87</v>
       </c>
       <c r="L26">
         <v>0</v>
       </c>
-      <c r="M26">
-        <v>216702</v>
-      </c>
-    </row>
-    <row r="27" spans="1:13">
+    </row>
+    <row r="27" spans="1:12">
       <c r="A27" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B27" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C27" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D27" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="E27" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F27">
         <v>64.29000000000001</v>
@@ -1820,30 +1741,27 @@
         <v>100.29</v>
       </c>
       <c r="K27" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="L27">
         <v>0</v>
       </c>
-      <c r="M27">
-        <v>216786</v>
-      </c>
-    </row>
-    <row r="28" spans="1:13">
+    </row>
+    <row r="28" spans="1:12">
       <c r="A28" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B28" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C28" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="D28" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="E28" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="F28">
         <v>26</v>
@@ -1861,30 +1779,27 @@
         <v>38.74</v>
       </c>
       <c r="K28" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="L28">
         <v>0</v>
       </c>
-      <c r="M28">
-        <v>126388</v>
-      </c>
-    </row>
-    <row r="29" spans="1:13">
+    </row>
+    <row r="29" spans="1:12">
       <c r="A29" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B29" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C29" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D29" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="E29" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="F29">
         <v>61.95</v>
@@ -1907,11 +1822,8 @@
       <c r="L29">
         <v>0</v>
       </c>
-      <c r="M29">
-        <v>126397</v>
-      </c>
-    </row>
-    <row r="32" spans="1:13">
+    </row>
+    <row r="32" spans="1:12">
       <c r="A32" s="3" t="s">
         <v>91</v>
       </c>
@@ -1943,7 +1855,7 @@
     </row>
     <row r="34" spans="1:6">
       <c r="A34" s="5" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="B34" s="6">
         <v>750.34</v>
@@ -1963,7 +1875,7 @@
     </row>
     <row r="35" spans="1:6">
       <c r="A35" s="5" t="s">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="B35" s="6">
         <v>408.62</v>
@@ -1983,7 +1895,7 @@
     </row>
     <row r="36" spans="1:6">
       <c r="A36" s="5" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="B36" s="6">
         <v>128.83</v>
@@ -1992,10 +1904,10 @@
         <v>2</v>
       </c>
       <c r="D36" s="7">
-        <v>1.7748</v>
+        <v>1.7448</v>
       </c>
       <c r="E36" s="6">
-        <v>228.65</v>
+        <v>224.78</v>
       </c>
       <c r="F36" s="6">
         <v>228.65</v>
@@ -2003,7 +1915,7 @@
     </row>
     <row r="37" spans="1:6">
       <c r="A37" s="5" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B37" s="6">
         <v>67.44</v>
@@ -2033,7 +1945,7 @@
       </c>
       <c r="D38" s="7"/>
       <c r="E38" s="9">
-        <v>1999.99</v>
+        <v>1996.12</v>
       </c>
       <c r="F38" s="9">
         <v>2035.41</v>

</xml_diff>